<commit_message>
Committing & pushing for backup purposes
</commit_message>
<xml_diff>
--- a/Amoritization.xlsx
+++ b/Amoritization.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\Misc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git_Repositories\PubDev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{260672BF-7013-4874-A939-8F4B4AEC8A15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{154BB628-36EE-45FE-9544-D38456F642BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5025" yWindow="1755" windowWidth="28770" windowHeight="16260" xr2:uid="{AE14A5DA-5418-4CB2-B16F-47804216F2DB}"/>
+    <workbookView xWindow="3840" yWindow="1575" windowWidth="24360" windowHeight="16905" xr2:uid="{AE14A5DA-5418-4CB2-B16F-47804216F2DB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -243,7 +243,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -280,7 +280,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -647,15 +646,18 @@
         <v>10000</v>
       </c>
       <c r="C2" s="10">
-        <f>A2</f>
-        <v>3.5999999999999997E-2</v>
+        <f>A3</f>
+        <v>0.1</v>
       </c>
       <c r="D2" s="11">
         <f>C2/12</f>
-        <v>2.9999999999999996E-3</v>
+        <v>8.3333333333333332E-3</v>
       </c>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A3" s="10">
+        <v>0.1</v>
+      </c>
       <c r="E3" s="11"/>
     </row>
     <row r="4" spans="1:20" ht="17.25" x14ac:dyDescent="0.3">
@@ -729,67 +731,67 @@
       </c>
       <c r="C6" s="17">
         <f>B2*(1+D2)</f>
-        <v>10029.999999999998</v>
+        <v>10083.333333333334</v>
       </c>
       <c r="D6" s="17">
         <f>B2*D2</f>
-        <v>29.999999999999996</v>
+        <v>83.333333333333329</v>
       </c>
       <c r="E6" s="18">
         <f>C6-B2</f>
-        <v>29.999999999998181</v>
+        <v>83.33333333333394</v>
       </c>
       <c r="F6" s="16">
         <v>13</v>
       </c>
       <c r="G6" s="17">
         <f>C17*(1+D2)</f>
-        <v>10397.097802289942</v>
+        <v>11139.190096699742</v>
       </c>
       <c r="H6" s="17">
         <f>C17*D2</f>
-        <v>31.097999408643894</v>
+        <v>92.059422286774719</v>
       </c>
       <c r="I6" s="18">
         <f>G6-B2</f>
-        <v>397.09780228994168</v>
-      </c>
-      <c r="J6" s="4">
+        <v>1139.1900966997418</v>
+      </c>
+      <c r="J6" s="16">
         <v>25</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="17">
         <f>G17*(1+D2)</f>
-        <v>10777.631376907515</v>
-      </c>
-      <c r="L6" s="1">
+        <v>12305.608860536884</v>
+      </c>
+      <c r="L6" s="17">
         <f>G17*D2</f>
-        <v>32.236185574000544</v>
-      </c>
-      <c r="M6" s="5">
+        <v>101.69924678129657</v>
+      </c>
+      <c r="M6" s="18">
         <f>K6-B2</f>
-        <v>777.631376907515</v>
+        <v>2305.6088605368841</v>
       </c>
       <c r="N6" s="3">
         <v>37</v>
       </c>
       <c r="O6" s="1">
         <f>K17*(1+D2)</f>
-        <v>11172.092472855062</v>
+        <v>13594.1669110565</v>
       </c>
       <c r="P6" s="1">
         <f>K17*D2</f>
-        <v>33.416029330573465</v>
+        <v>112.34848686823554</v>
       </c>
       <c r="Q6" s="5">
         <f>O6-B2</f>
-        <v>1172.0924728550617</v>
+        <v>3594.1669110564999</v>
       </c>
       <c r="S6" s="6" t="s">
         <v>1</v>
       </c>
       <c r="T6" s="7">
         <f>O6-B2</f>
-        <v>1172.0924728550617</v>
+        <v>3594.1669110564999</v>
       </c>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.25">
@@ -801,56 +803,56 @@
       </c>
       <c r="C7" s="17">
         <f>C6*(1+D2)</f>
-        <v>10060.089999999997</v>
+        <v>10167.361111111111</v>
       </c>
       <c r="D7" s="17">
         <f>C6*D2</f>
-        <v>30.089999999999989</v>
+        <v>84.027777777777786</v>
       </c>
       <c r="E7" s="18">
         <f>C7-B2</f>
-        <v>60.089999999996508</v>
+        <v>167.36111111111131</v>
       </c>
       <c r="F7" s="19">
         <v>14</v>
       </c>
       <c r="G7" s="17">
         <f>G6*(1+D2)</f>
-        <v>10428.289095696811</v>
+        <v>11232.016680838906</v>
       </c>
       <c r="H7" s="17">
         <f>G6*D2</f>
-        <v>31.191293406869821</v>
+        <v>92.82658413916451</v>
       </c>
       <c r="I7" s="18">
         <f>G7-B2</f>
-        <v>428.28909569681127</v>
+        <v>1232.0166808389058</v>
       </c>
       <c r="J7" s="3">
         <v>26</v>
       </c>
       <c r="K7" s="1">
         <f>K6*(1+D2)</f>
-        <v>10809.964271038236</v>
+        <v>12408.155601041357</v>
       </c>
       <c r="L7" s="1">
         <f>K6*D2</f>
-        <v>32.332894130722543</v>
+        <v>102.54674050447403</v>
       </c>
       <c r="M7" s="5">
         <f>K7-B2</f>
-        <v>809.96427103823589</v>
-      </c>
-      <c r="N7" s="22"/>
-      <c r="O7" s="22"/>
-      <c r="P7" s="22"/>
-      <c r="Q7" s="22"/>
+        <v>2408.1556010413569</v>
+      </c>
+      <c r="N7" s="1"/>
+      <c r="O7" s="1"/>
+      <c r="P7" s="1"/>
+      <c r="Q7" s="1"/>
       <c r="S7" s="15" t="s">
         <v>5</v>
       </c>
       <c r="T7" s="5">
         <f>B2+T6</f>
-        <v>11172.092472855062</v>
+        <v>13594.1669110565</v>
       </c>
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.25">
@@ -862,56 +864,56 @@
       </c>
       <c r="C8" s="17">
         <f>C7*(1+D2)</f>
-        <v>10090.270269999995</v>
+        <v>10252.08912037037</v>
       </c>
       <c r="D8" s="17">
         <f>C7*D2</f>
-        <v>30.180269999999986</v>
+        <v>84.728009259259267</v>
       </c>
       <c r="E8" s="18">
         <f>C8-B2</f>
-        <v>90.270269999995435</v>
+        <v>252.08912037037044</v>
       </c>
       <c r="F8" s="19">
         <v>15</v>
       </c>
       <c r="G8" s="17">
         <f>G7*(1+D2)</f>
-        <v>10459.573962983901</v>
+        <v>11325.616819845896</v>
       </c>
       <c r="H8" s="17">
         <f>G7*D2</f>
-        <v>31.284867287090432</v>
+        <v>93.600139006990887</v>
       </c>
       <c r="I8" s="18">
         <f>G8-B2</f>
-        <v>459.57396298390086</v>
+        <v>1325.6168198458963</v>
       </c>
       <c r="J8" s="3">
         <v>27</v>
       </c>
       <c r="K8" s="1">
         <f>K7*(1+D2)</f>
-        <v>10842.39416385135</v>
+        <v>12511.5568977167</v>
       </c>
       <c r="L8" s="1">
         <f>K7*D2</f>
-        <v>32.429892813114705</v>
+        <v>103.40129667534464</v>
       </c>
       <c r="M8" s="5">
         <f>K8-B2</f>
-        <v>842.39416385134973</v>
-      </c>
-      <c r="N8" s="22"/>
-      <c r="O8" s="22"/>
-      <c r="P8" s="22"/>
-      <c r="Q8" s="22"/>
+        <v>2511.5568977167004</v>
+      </c>
+      <c r="N8" s="1"/>
+      <c r="O8" s="1"/>
+      <c r="P8" s="1"/>
+      <c r="Q8" s="1"/>
       <c r="S8" s="15" t="s">
         <v>6</v>
       </c>
       <c r="T8" s="5">
         <f>T7-B2</f>
-        <v>1172.0924728550617</v>
+        <v>3594.1669110564999</v>
       </c>
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.25">
@@ -923,56 +925,56 @@
       </c>
       <c r="C9" s="17">
         <f>C8*(1+D2)</f>
-        <v>10120.541080809995</v>
+        <v>10337.523196373457</v>
       </c>
       <c r="D9" s="17">
         <f>C8*D2</f>
-        <v>30.270810809999983</v>
+        <v>85.434076003086417</v>
       </c>
       <c r="E9" s="18">
         <f>C9-B2</f>
-        <v>120.54108080999504</v>
+        <v>337.52319637345681</v>
       </c>
       <c r="F9" s="19">
         <v>16</v>
       </c>
       <c r="G9" s="17">
         <f>G8*(1+D2)</f>
-        <v>10490.952684872851</v>
+        <v>11419.996960011278</v>
       </c>
       <c r="H9" s="17">
         <f>G8*D2</f>
-        <v>31.378721888951699</v>
+        <v>94.380140165382471</v>
       </c>
       <c r="I9" s="18">
         <f>G9-B2</f>
-        <v>490.95268487285102</v>
+        <v>1419.9969600112781</v>
       </c>
       <c r="J9" s="3">
         <v>28</v>
       </c>
       <c r="K9" s="1">
         <f>K8*(1+D2)</f>
-        <v>10874.921346342902</v>
+        <v>12615.81987186434</v>
       </c>
       <c r="L9" s="1">
         <f>K8*D2</f>
-        <v>32.527182491554044</v>
+        <v>104.26297414763917</v>
       </c>
       <c r="M9" s="5">
         <f>K9-B2</f>
-        <v>874.92134634290232</v>
-      </c>
-      <c r="N9" s="22"/>
-      <c r="O9" s="22"/>
-      <c r="P9" s="22"/>
-      <c r="Q9" s="22"/>
+        <v>2615.8198718643398</v>
+      </c>
+      <c r="N9" s="1"/>
+      <c r="O9" s="1"/>
+      <c r="P9" s="1"/>
+      <c r="Q9" s="1"/>
       <c r="S9" s="8" t="s">
         <v>19</v>
       </c>
       <c r="T9" s="9">
         <f>B2-T8</f>
-        <v>8827.9075271449383</v>
+        <v>6405.8330889435001</v>
       </c>
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.25">
@@ -984,50 +986,50 @@
       </c>
       <c r="C10" s="17">
         <f>C9*(1+D2)</f>
-        <v>10150.902704052423</v>
+        <v>10423.669223009902</v>
       </c>
       <c r="D10" s="17">
         <f>C9*D2</f>
-        <v>30.361623242429982</v>
+        <v>86.14602663644547</v>
       </c>
       <c r="E10" s="18">
         <f>C10-B2</f>
-        <v>150.90270405242336</v>
+        <v>423.66922300990154</v>
       </c>
       <c r="F10" s="19">
         <v>17</v>
       </c>
       <c r="G10" s="17">
         <f>G9*(1+D2)</f>
-        <v>10522.425542927469</v>
+        <v>11515.163601344706</v>
       </c>
       <c r="H10" s="17">
         <f>G9*D2</f>
-        <v>31.472858054618548</v>
+        <v>95.166641333427322</v>
       </c>
       <c r="I10" s="18">
         <f>G10-B2</f>
-        <v>522.425542927469</v>
+        <v>1515.163601344706</v>
       </c>
       <c r="J10" s="3">
         <v>19</v>
       </c>
       <c r="K10" s="1">
         <f>K9*(1+D2)</f>
-        <v>10907.546110381931</v>
+        <v>12720.951704129875</v>
       </c>
       <c r="L10" s="1">
         <f>K9*D2</f>
-        <v>32.624764039028705</v>
+        <v>105.13183226553616</v>
       </c>
       <c r="M10" s="5">
         <f>K10-B2</f>
-        <v>907.5461103819307</v>
-      </c>
-      <c r="N10" s="22"/>
-      <c r="O10" s="22"/>
-      <c r="P10" s="22"/>
-      <c r="Q10" s="22"/>
+        <v>2720.951704129875</v>
+      </c>
+      <c r="N10" s="1"/>
+      <c r="O10" s="1"/>
+      <c r="P10" s="1"/>
+      <c r="Q10" s="1"/>
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
@@ -1038,50 +1040,50 @@
       </c>
       <c r="C11" s="17">
         <f>C10*(1+D2)</f>
-        <v>10181.355412164579</v>
+        <v>10510.53313320165</v>
       </c>
       <c r="D11" s="17">
         <f>C10*D2</f>
-        <v>30.452708112157268</v>
+        <v>86.863910191749184</v>
       </c>
       <c r="E11" s="18">
         <f>C11-B2</f>
-        <v>181.35541216457932</v>
+        <v>510.53313320165034</v>
       </c>
       <c r="F11" s="19">
         <v>18</v>
       </c>
       <c r="G11" s="17">
         <f>G10*(1+D2)</f>
-        <v>10553.99281955625</v>
+        <v>11611.123298022578</v>
       </c>
       <c r="H11" s="17">
         <f>G10*D2</f>
-        <v>31.567276628782402</v>
+        <v>95.959696677872543</v>
       </c>
       <c r="I11" s="18">
         <f>G11-B2</f>
-        <v>553.99281955624974</v>
+        <v>1611.1232980225777</v>
       </c>
       <c r="J11" s="3">
         <v>30</v>
       </c>
       <c r="K11" s="1">
         <f>K10*(1+D2)</f>
-        <v>10940.268748713075</v>
+        <v>12826.959634997624</v>
       </c>
       <c r="L11" s="1">
         <f>K10*D2</f>
-        <v>32.722638331145788</v>
+        <v>106.00793086774895</v>
       </c>
       <c r="M11" s="5">
         <f>K11-B2</f>
-        <v>940.26874871307518</v>
-      </c>
-      <c r="N11" s="22"/>
-      <c r="O11" s="22"/>
-      <c r="P11" s="22"/>
-      <c r="Q11" s="22"/>
+        <v>2826.9596349976237</v>
+      </c>
+      <c r="N11" s="1"/>
+      <c r="O11" s="1"/>
+      <c r="P11" s="1"/>
+      <c r="Q11" s="1"/>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
@@ -1092,50 +1094,50 @@
       </c>
       <c r="C12" s="17">
         <f>C11*(1+D2)</f>
-        <v>10211.899478401072</v>
+        <v>10598.120909311663</v>
       </c>
       <c r="D12" s="17">
         <f>C11*D2</f>
-        <v>30.544066236493734</v>
+        <v>87.587776110013749</v>
       </c>
       <c r="E12" s="18">
         <f>C12-B2</f>
-        <v>211.89947840107197</v>
+        <v>598.12090931166313</v>
       </c>
       <c r="F12" s="19">
         <v>19</v>
       </c>
       <c r="G12" s="17">
         <f>G11*(1+D2)</f>
-        <v>10585.654798014917</v>
+        <v>11707.882658839431</v>
       </c>
       <c r="H12" s="17">
         <f>G11*D2</f>
-        <v>31.661978458668745</v>
+        <v>96.759360816854809</v>
       </c>
       <c r="I12" s="18">
         <f>G12-B2</f>
-        <v>585.65479801491711</v>
+        <v>1707.8826588394313</v>
       </c>
       <c r="J12" s="3">
         <v>31</v>
       </c>
       <c r="K12" s="1">
         <f>K11*(1+D2)</f>
-        <v>10973.089554959213</v>
+        <v>12933.85096528927</v>
       </c>
       <c r="L12" s="1">
         <f>K11*D2</f>
-        <v>32.82080624613922</v>
+        <v>106.89133029164687</v>
       </c>
       <c r="M12" s="5">
         <f>K12-B2</f>
-        <v>973.08955495921327</v>
-      </c>
-      <c r="N12" s="22"/>
-      <c r="O12" s="22"/>
-      <c r="P12" s="22"/>
-      <c r="Q12" s="22"/>
+        <v>2933.8509652892699</v>
+      </c>
+      <c r="N12" s="1"/>
+      <c r="O12" s="1"/>
+      <c r="P12" s="1"/>
+      <c r="Q12" s="1"/>
     </row>
     <row r="13" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
@@ -1146,50 +1148,50 @@
       </c>
       <c r="C13" s="17">
         <f>C12*(1+D2)</f>
-        <v>10242.535176836274</v>
+        <v>10686.438583555926</v>
       </c>
       <c r="D13" s="17">
         <f>C12*D2</f>
-        <v>30.635698435203214</v>
+        <v>88.317674244263856</v>
       </c>
       <c r="E13" s="18">
         <f>C13-B2</f>
-        <v>242.53517683627433</v>
+        <v>686.43858355592602</v>
       </c>
       <c r="F13" s="19">
         <v>20</v>
       </c>
       <c r="G13" s="17">
         <f>G12*(1+D2)</f>
-        <v>10617.411762408961</v>
+        <v>11805.448347663092</v>
       </c>
       <c r="H13" s="17">
         <f>G12*D2</f>
-        <v>31.756964394044747</v>
+        <v>97.56568882366193</v>
       </c>
       <c r="I13" s="18">
         <f>G13-B2</f>
-        <v>617.41176240896129</v>
+        <v>1805.4483476630921</v>
       </c>
       <c r="J13" s="3">
         <v>32</v>
       </c>
       <c r="K13" s="1">
         <f>K12*(1+D2)</f>
-        <v>11006.00882362409</v>
+        <v>13041.63305666668</v>
       </c>
       <c r="L13" s="1">
         <f>K12*D2</f>
-        <v>32.919268664877634</v>
+        <v>107.78209137741058</v>
       </c>
       <c r="M13" s="5">
         <f>K13-B2</f>
-        <v>1006.0088236240899</v>
-      </c>
-      <c r="N13" s="22"/>
-      <c r="O13" s="22"/>
-      <c r="P13" s="22"/>
-      <c r="Q13" s="22"/>
+        <v>3041.6330566666802</v>
+      </c>
+      <c r="N13" s="1"/>
+      <c r="O13" s="1"/>
+      <c r="P13" s="1"/>
+      <c r="Q13" s="1"/>
     </row>
     <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
@@ -1200,50 +1202,50 @@
       </c>
       <c r="C14" s="17">
         <f>C13*(1+D2)</f>
-        <v>10273.262782366783</v>
+        <v>10775.492238418892</v>
       </c>
       <c r="D14" s="17">
         <f>C13*D2</f>
-        <v>30.727605530508818</v>
+        <v>89.053654862966056</v>
       </c>
       <c r="E14" s="18">
         <f>C14-B2</f>
-        <v>273.26278236678263</v>
+        <v>775.49223841889216</v>
       </c>
       <c r="F14" s="19">
         <v>21</v>
       </c>
       <c r="G14" s="17">
         <f>G13*(1+D2)</f>
-        <v>10649.263997696187</v>
+        <v>11903.827083893617</v>
       </c>
       <c r="H14" s="17">
         <f>G13*D2</f>
-        <v>31.852235287226879</v>
+        <v>98.37873623052576</v>
       </c>
       <c r="I14" s="18">
         <f>G14-B2</f>
-        <v>649.26399769618729</v>
+        <v>1903.8270838936169</v>
       </c>
       <c r="J14" s="3">
         <v>33</v>
       </c>
       <c r="K14" s="1">
         <f>K13*(1+D2)</f>
-        <v>11039.026850094961</v>
+        <v>13150.313332138901</v>
       </c>
       <c r="L14" s="1">
         <f>K13*D2</f>
-        <v>33.018026470872265</v>
+        <v>108.68027547222233</v>
       </c>
       <c r="M14" s="5">
         <f>K14-B2</f>
-        <v>1039.0268500949605</v>
-      </c>
-      <c r="N14" s="22"/>
-      <c r="O14" s="22"/>
-      <c r="P14" s="22"/>
-      <c r="Q14" s="22"/>
+        <v>3150.3133321389014</v>
+      </c>
+      <c r="N14" s="1"/>
+      <c r="O14" s="1"/>
+      <c r="P14" s="1"/>
+      <c r="Q14" s="1"/>
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
@@ -1254,50 +1256,50 @@
       </c>
       <c r="C15" s="17">
         <f>C14*(1+D2)</f>
-        <v>10304.082570713881</v>
+        <v>10865.288007072382</v>
       </c>
       <c r="D15" s="17">
         <f>C14*D2</f>
-        <v>30.819788347100346</v>
+        <v>89.795768653490768</v>
       </c>
       <c r="E15" s="18">
         <f>C15-B2</f>
-        <v>304.08257071388107</v>
+        <v>865.28800707238224</v>
       </c>
       <c r="F15" s="19">
         <v>22</v>
       </c>
       <c r="G15" s="17">
         <f>G14*(1+D2)</f>
-        <v>10681.211789689274</v>
+        <v>12003.025642926063</v>
       </c>
       <c r="H15" s="17">
         <f>G14*D2</f>
-        <v>31.947791993088558</v>
+        <v>99.198559032446809</v>
       </c>
       <c r="I15" s="18">
         <f>G15-B2</f>
-        <v>681.21178968927416</v>
+        <v>2003.0256429260626</v>
       </c>
       <c r="J15" s="3">
         <v>34</v>
       </c>
       <c r="K15" s="1">
         <f>K14*(1+D2)</f>
-        <v>11072.143930645245</v>
+        <v>13259.899276573391</v>
       </c>
       <c r="L15" s="1">
         <f>K14*D2</f>
-        <v>33.117080550284875</v>
+        <v>109.58594443449084</v>
       </c>
       <c r="M15" s="5">
         <f>K15-B2</f>
-        <v>1072.1439306452448</v>
-      </c>
-      <c r="N15" s="22"/>
-      <c r="O15" s="22"/>
-      <c r="P15" s="22"/>
-      <c r="Q15" s="22"/>
+        <v>3259.899276573391</v>
+      </c>
+      <c r="N15" s="1"/>
+      <c r="O15" s="1"/>
+      <c r="P15" s="1"/>
+      <c r="Q15" s="1"/>
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
@@ -1308,50 +1310,50 @@
       </c>
       <c r="C16" s="17">
         <f>C15*(1+D2)</f>
-        <v>10334.994818426021</v>
+        <v>10955.832073797985</v>
       </c>
       <c r="D16" s="17">
         <f>C15*D2</f>
-        <v>30.912247712141639</v>
+        <v>90.544066725603187</v>
       </c>
       <c r="E16" s="18">
         <f>C16-B2</f>
-        <v>334.99481842602108</v>
+        <v>955.83207379798478</v>
       </c>
       <c r="F16" s="19">
         <v>23</v>
       </c>
       <c r="G16" s="17">
         <f>G15*(1+D2)</f>
-        <v>10713.255425058342</v>
+        <v>12103.050856617112</v>
       </c>
       <c r="H16" s="17">
         <f>G15*D2</f>
-        <v>32.043635369067822</v>
+        <v>100.02521369105052</v>
       </c>
       <c r="I16" s="18">
         <f>G16-B2</f>
-        <v>713.25542505834164</v>
+        <v>2103.050856617112</v>
       </c>
       <c r="J16" s="3">
         <v>35</v>
       </c>
       <c r="K16" s="1">
         <f>K15*(1+D2)</f>
-        <v>11105.360362437179</v>
+        <v>13370.398437211503</v>
       </c>
       <c r="L16" s="1">
         <f>K15*D2</f>
-        <v>33.216431791935733</v>
+        <v>110.49916063811159</v>
       </c>
       <c r="M16" s="5">
         <f>K16-B2</f>
-        <v>1105.360362437179</v>
-      </c>
-      <c r="N16" s="22"/>
-      <c r="O16" s="22"/>
-      <c r="P16" s="22"/>
-      <c r="Q16" s="22"/>
+        <v>3370.3984372115028</v>
+      </c>
+      <c r="N16" s="1"/>
+      <c r="O16" s="1"/>
+      <c r="P16" s="1"/>
+      <c r="Q16" s="1"/>
     </row>
     <row r="17" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
@@ -1362,50 +1364,50 @@
       </c>
       <c r="C17" s="17">
         <f>C16*(1+D2)</f>
-        <v>10365.999802881299</v>
+        <v>11047.130674412967</v>
       </c>
       <c r="D17" s="17">
         <f>C16*D2</f>
-        <v>31.004984455278059</v>
+        <v>91.298600614983201</v>
       </c>
       <c r="E17" s="18">
         <f>C17-B2</f>
-        <v>365.99980288129882</v>
+        <v>1047.130674412967</v>
       </c>
       <c r="F17" s="19">
         <v>24</v>
       </c>
       <c r="G17" s="17">
         <f>G16*(1+D2)</f>
-        <v>10745.395191333515</v>
+        <v>12203.909613755588</v>
       </c>
       <c r="H17" s="17">
         <f>G16*D2</f>
-        <v>32.13976627517502</v>
+        <v>100.85875713847594</v>
       </c>
       <c r="I17" s="18">
         <f>G17-B2</f>
-        <v>745.39519133351496</v>
+        <v>2203.909613755588</v>
       </c>
       <c r="J17" s="3">
         <v>36</v>
       </c>
       <c r="K17" s="1">
         <f>K16*(1+D2)</f>
-        <v>11138.67644352449</v>
+        <v>13481.818424188265</v>
       </c>
       <c r="L17" s="1">
         <f>K16*D2</f>
-        <v>33.316081087311531</v>
+        <v>111.41998697676252</v>
       </c>
       <c r="M17" s="5">
         <f>K17-B2</f>
-        <v>1138.6764435244895</v>
-      </c>
-      <c r="N17" s="22"/>
-      <c r="O17" s="22"/>
-      <c r="P17" s="22"/>
-      <c r="Q17" s="22"/>
+        <v>3481.8184241882645</v>
+      </c>
+      <c r="N17" s="1"/>
+      <c r="O17" s="1"/>
+      <c r="P17" s="1"/>
+      <c r="Q17" s="1"/>
     </row>
     <row r="18" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A18" s="14"/>
@@ -1578,15 +1580,15 @@
       <c r="N23" s="3">
         <v>37</v>
       </c>
-      <c r="O23" s="22">
+      <c r="O23" s="1">
         <f>K34*(1+D20)</f>
         <v>44688.369891420247</v>
       </c>
-      <c r="P23" s="22">
+      <c r="P23" s="1">
         <f>K34*D20</f>
         <v>133.66411732229386</v>
       </c>
-      <c r="Q23" s="22">
+      <c r="Q23" s="1">
         <f>O23-B20</f>
         <v>4688.3698914202469</v>
       </c>
@@ -1644,10 +1646,10 @@
         <f>K24-B20</f>
         <v>3239.8570841529436</v>
       </c>
-      <c r="N24" s="22"/>
-      <c r="O24" s="22"/>
-      <c r="P24" s="22"/>
-      <c r="Q24" s="22"/>
+      <c r="N24" s="1"/>
+      <c r="O24" s="1"/>
+      <c r="P24" s="1"/>
+      <c r="Q24" s="1"/>
       <c r="S24" s="15" t="s">
         <v>5</v>
       </c>
@@ -1702,10 +1704,10 @@
         <f>K25-B20</f>
         <v>3369.5766554053989</v>
       </c>
-      <c r="N25" s="22"/>
-      <c r="O25" s="22"/>
-      <c r="P25" s="22"/>
-      <c r="Q25" s="22"/>
+      <c r="N25" s="1"/>
+      <c r="O25" s="1"/>
+      <c r="P25" s="1"/>
+      <c r="Q25" s="1"/>
       <c r="S25" s="15" t="s">
         <v>6</v>
       </c>
@@ -1760,10 +1762,10 @@
         <f>K26-B20</f>
         <v>3499.6853853716093</v>
       </c>
-      <c r="N26" s="22"/>
-      <c r="O26" s="22"/>
-      <c r="P26" s="22"/>
-      <c r="Q26" s="22"/>
+      <c r="N26" s="1"/>
+      <c r="O26" s="1"/>
+      <c r="P26" s="1"/>
+      <c r="Q26" s="1"/>
       <c r="S26" s="8" t="s">
         <v>19</v>
       </c>
@@ -1818,10 +1820,10 @@
         <f>K27-B20</f>
         <v>3630.1844415277228</v>
       </c>
-      <c r="N27" s="22"/>
-      <c r="O27" s="22"/>
-      <c r="P27" s="22"/>
-      <c r="Q27" s="22"/>
+      <c r="N27" s="1"/>
+      <c r="O27" s="1"/>
+      <c r="P27" s="1"/>
+      <c r="Q27" s="1"/>
     </row>
     <row r="28" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B28" s="3">
@@ -1869,10 +1871,10 @@
         <f>K28-B20</f>
         <v>3761.0749948523007</v>
       </c>
-      <c r="N28" s="22"/>
-      <c r="O28" s="22"/>
-      <c r="P28" s="22"/>
-      <c r="Q28" s="22"/>
+      <c r="N28" s="1"/>
+      <c r="O28" s="1"/>
+      <c r="P28" s="1"/>
+      <c r="Q28" s="1"/>
     </row>
     <row r="29" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B29" s="3">
@@ -1920,10 +1922,10 @@
         <f>K29-B20</f>
         <v>3892.3582198368531</v>
       </c>
-      <c r="N29" s="22"/>
-      <c r="O29" s="22"/>
-      <c r="P29" s="22"/>
-      <c r="Q29" s="22"/>
+      <c r="N29" s="1"/>
+      <c r="O29" s="1"/>
+      <c r="P29" s="1"/>
+      <c r="Q29" s="1"/>
     </row>
     <row r="30" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B30" s="3">
@@ -1971,10 +1973,10 @@
         <f>K30-B20</f>
         <v>4024.0352944963597</v>
       </c>
-      <c r="N30" s="22"/>
-      <c r="O30" s="22"/>
-      <c r="P30" s="22"/>
-      <c r="Q30" s="22"/>
+      <c r="N30" s="1"/>
+      <c r="O30" s="1"/>
+      <c r="P30" s="1"/>
+      <c r="Q30" s="1"/>
     </row>
     <row r="31" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B31" s="3">
@@ -2022,10 +2024,10 @@
         <f>K31-B20</f>
         <v>4156.1074003798421</v>
       </c>
-      <c r="N31" s="22"/>
-      <c r="O31" s="22"/>
-      <c r="P31" s="22"/>
-      <c r="Q31" s="22"/>
+      <c r="N31" s="1"/>
+      <c r="O31" s="1"/>
+      <c r="P31" s="1"/>
+      <c r="Q31" s="1"/>
     </row>
     <row r="32" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B32" s="3">
@@ -2073,10 +2075,10 @@
         <f>K32-B20</f>
         <v>4288.5757225809793</v>
       </c>
-      <c r="N32" s="22"/>
-      <c r="O32" s="22"/>
-      <c r="P32" s="22"/>
-      <c r="Q32" s="22"/>
+      <c r="N32" s="1"/>
+      <c r="O32" s="1"/>
+      <c r="P32" s="1"/>
+      <c r="Q32" s="1"/>
     </row>
     <row r="33" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B33" s="3">
@@ -2124,10 +2126,10 @@
         <f>K33-B20</f>
         <v>4421.441449748716</v>
       </c>
-      <c r="N33" s="22"/>
-      <c r="O33" s="22"/>
-      <c r="P33" s="22"/>
-      <c r="Q33" s="22"/>
+      <c r="N33" s="1"/>
+      <c r="O33" s="1"/>
+      <c r="P33" s="1"/>
+      <c r="Q33" s="1"/>
     </row>
     <row r="34" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B34" s="3">
@@ -2175,10 +2177,10 @@
         <f>K34-B20</f>
         <v>4554.7057740979581</v>
       </c>
-      <c r="N34" s="22"/>
-      <c r="O34" s="22"/>
-      <c r="P34" s="22"/>
-      <c r="Q34" s="22"/>
+      <c r="N34" s="1"/>
+      <c r="O34" s="1"/>
+      <c r="P34" s="1"/>
+      <c r="Q34" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>